<commit_message>
Ajout LazyPredict + SHAP pour 4 modeles sans consomixte
</commit_message>
<xml_diff>
--- a/notebooks/LazyPredict_resultats.xlsx
+++ b/notebooks/LazyPredict_resultats.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.9997</v>
+        <v>0.9813</v>
       </c>
       <c r="C2" t="n">
-        <v>0.9997</v>
+        <v>0.9814000000000001</v>
       </c>
       <c r="D2" t="n">
-        <v>0.6046</v>
+        <v>4.6883</v>
       </c>
       <c r="E2" t="n">
-        <v>3.2585</v>
+        <v>3.2252</v>
       </c>
     </row>
     <row r="3">
@@ -469,700 +469,700 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.9991</v>
+        <v>0.9782</v>
       </c>
       <c r="C3" t="n">
-        <v>0.9991</v>
+        <v>0.9784</v>
       </c>
       <c r="D3" t="n">
-        <v>1.0046</v>
+        <v>5.0573</v>
       </c>
       <c r="E3" t="n">
-        <v>4.9814</v>
+        <v>4.7196</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BaggingRegressor</t>
+          <t>DecisionTreeRegressor</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.9989</v>
+        <v>0.9769</v>
       </c>
       <c r="C4" t="n">
-        <v>0.9989</v>
+        <v>0.9771</v>
       </c>
       <c r="D4" t="n">
-        <v>1.1529</v>
+        <v>5.2098</v>
       </c>
       <c r="E4" t="n">
-        <v>0.5639</v>
+        <v>0.1036</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ExtraTreeRegressor</t>
+          <t>BaggingRegressor</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.9985000000000001</v>
+        <v>0.9761</v>
       </c>
       <c r="C5" t="n">
-        <v>0.9985000000000001</v>
+        <v>0.9762999999999999</v>
       </c>
       <c r="D5" t="n">
-        <v>1.3411</v>
+        <v>5.2933</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0675</v>
+        <v>0.512</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DecisionTreeRegressor</t>
+          <t>ExtraTreeRegressor</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.9983</v>
+        <v>0.9754</v>
       </c>
       <c r="C6" t="n">
-        <v>0.9983</v>
+        <v>0.9756</v>
       </c>
       <c r="D6" t="n">
-        <v>1.4302</v>
+        <v>5.3691</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1131</v>
+        <v>0.0766</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MLPRegressor</t>
+          <t>HistGradientBoostingRegressor</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.9979</v>
+        <v>0.9707</v>
       </c>
       <c r="C7" t="n">
-        <v>0.998</v>
+        <v>0.9709</v>
       </c>
       <c r="D7" t="n">
-        <v>1.5547</v>
+        <v>5.8678</v>
       </c>
       <c r="E7" t="n">
-        <v>7.7383</v>
+        <v>2.0487</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GradientBoostingRegressor</t>
+          <t>MLPRegressor</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.9976</v>
+        <v>0.9624</v>
       </c>
       <c r="C8" t="n">
-        <v>0.9976</v>
+        <v>0.9627</v>
       </c>
       <c r="D8" t="n">
-        <v>1.6711</v>
+        <v>6.6418</v>
       </c>
       <c r="E8" t="n">
-        <v>3.0885</v>
+        <v>11.615</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>RidgeCV</t>
+          <t>KNeighborsRegressor</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.9972</v>
+        <v>0.9532</v>
       </c>
       <c r="C9" t="n">
-        <v>0.9973</v>
+        <v>0.9535</v>
       </c>
       <c r="D9" t="n">
-        <v>1.7984</v>
+        <v>7.4144</v>
       </c>
       <c r="E9" t="n">
-        <v>0.1535</v>
+        <v>1.0117</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Ridge</t>
+          <t>GradientBoostingRegressor</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.9972</v>
+        <v>0.9487</v>
       </c>
       <c r="C10" t="n">
-        <v>0.9973</v>
+        <v>0.9492</v>
       </c>
       <c r="D10" t="n">
-        <v>1.7986</v>
+        <v>7.7555</v>
       </c>
       <c r="E10" t="n">
-        <v>0.0479</v>
+        <v>2.9046</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>BayesianRidge</t>
+          <t>PoissonRegressor</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.9972</v>
+        <v>0.868</v>
       </c>
       <c r="C11" t="n">
-        <v>0.9973</v>
+        <v>0.8691</v>
       </c>
       <c r="D11" t="n">
-        <v>1.7987</v>
+        <v>12.4442</v>
       </c>
       <c r="E11" t="n">
-        <v>0.1178</v>
+        <v>0.1451</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>LinearRegression</t>
+          <t>BayesianRidge</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.9972</v>
+        <v>0.8582</v>
       </c>
       <c r="C12" t="n">
-        <v>0.9973</v>
+        <v>0.8593</v>
       </c>
       <c r="D12" t="n">
-        <v>1.7987</v>
+        <v>12.8998</v>
       </c>
       <c r="E12" t="n">
-        <v>0.08890000000000001</v>
+        <v>0.1439</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TransformedTargetRegressor</t>
+          <t>RidgeCV</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.9972</v>
+        <v>0.8582</v>
       </c>
       <c r="C13" t="n">
-        <v>0.9973</v>
+        <v>0.8593</v>
       </c>
       <c r="D13" t="n">
-        <v>1.7987</v>
+        <v>12.8999</v>
       </c>
       <c r="E13" t="n">
-        <v>0.0847</v>
+        <v>0.1592</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>LassoLarsIC</t>
+          <t>Ridge</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.9972</v>
+        <v>0.8582</v>
       </c>
       <c r="C14" t="n">
-        <v>0.9973</v>
+        <v>0.8593</v>
       </c>
       <c r="D14" t="n">
-        <v>1.799</v>
+        <v>12.8999</v>
       </c>
       <c r="E14" t="n">
-        <v>0.1362</v>
+        <v>0.049</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>LassoLarsCV</t>
+          <t>LinearRegression</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.9972</v>
+        <v>0.8582</v>
       </c>
       <c r="C15" t="n">
-        <v>0.9973</v>
+        <v>0.8593</v>
       </c>
       <c r="D15" t="n">
-        <v>1.7992</v>
+        <v>12.8999</v>
       </c>
       <c r="E15" t="n">
-        <v>0.2302</v>
+        <v>0.0844</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>LassoCV</t>
+          <t>TransformedTargetRegressor</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.9971</v>
+        <v>0.8582</v>
       </c>
       <c r="C16" t="n">
-        <v>0.9972</v>
+        <v>0.8593</v>
       </c>
       <c r="D16" t="n">
-        <v>1.8343</v>
+        <v>12.8999</v>
       </c>
       <c r="E16" t="n">
-        <v>0.3204</v>
+        <v>0.0897</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>LarsCV</t>
+          <t>LassoCV</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.9971</v>
+        <v>0.8577</v>
       </c>
       <c r="C17" t="n">
-        <v>0.9971</v>
+        <v>0.8588</v>
       </c>
       <c r="D17" t="n">
-        <v>1.8422</v>
+        <v>12.9228</v>
       </c>
       <c r="E17" t="n">
-        <v>0.2462</v>
+        <v>0.3595</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>HistGradientBoostingRegressor</t>
+          <t>LarsCV</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.9965000000000001</v>
+        <v>0.857</v>
       </c>
       <c r="C18" t="n">
-        <v>0.9965000000000001</v>
+        <v>0.8582</v>
       </c>
       <c r="D18" t="n">
-        <v>2.0394</v>
+        <v>12.9544</v>
       </c>
       <c r="E18" t="n">
-        <v>2.1255</v>
+        <v>0.2895</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>HuberRegressor</t>
+          <t>ElasticNetCV</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.9961</v>
+        <v>0.8538</v>
       </c>
       <c r="C19" t="n">
-        <v>0.9961</v>
+        <v>0.855</v>
       </c>
       <c r="D19" t="n">
-        <v>2.1382</v>
+        <v>13.0991</v>
       </c>
       <c r="E19" t="n">
-        <v>0.7739</v>
+        <v>0.2254</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>OrthogonalMatchingPursuitCV</t>
+          <t>HuberRegressor</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.9961</v>
+        <v>0.8439</v>
       </c>
       <c r="C20" t="n">
-        <v>0.9961</v>
+        <v>0.8452</v>
       </c>
       <c r="D20" t="n">
-        <v>2.1449</v>
+        <v>13.5325</v>
       </c>
       <c r="E20" t="n">
-        <v>0.1406</v>
+        <v>0.8285</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>OrthogonalMatchingPursuit</t>
+          <t>LinearSVR</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.9961</v>
+        <v>0.838</v>
       </c>
       <c r="C21" t="n">
-        <v>0.9961</v>
+        <v>0.8393</v>
       </c>
       <c r="D21" t="n">
-        <v>2.1449</v>
+        <v>13.7868</v>
       </c>
       <c r="E21" t="n">
-        <v>0.0466</v>
+        <v>8.2089</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>LinearSVR</t>
+          <t>LassoLarsCV</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.9959</v>
+        <v>0.8329</v>
       </c>
       <c r="C22" t="n">
-        <v>0.9959</v>
+        <v>0.8343</v>
       </c>
       <c r="D22" t="n">
-        <v>2.2062</v>
+        <v>14.002</v>
       </c>
       <c r="E22" t="n">
-        <v>8.7966</v>
+        <v>0.2513</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ElasticNetCV</t>
+          <t>LassoLarsIC</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0.9933999999999999</v>
+        <v>0.8329</v>
       </c>
       <c r="C23" t="n">
-        <v>0.9935</v>
+        <v>0.8343</v>
       </c>
       <c r="D23" t="n">
-        <v>2.7807</v>
+        <v>14.002</v>
       </c>
       <c r="E23" t="n">
-        <v>0.1718</v>
+        <v>0.1227</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>RANSACRegressor</t>
+          <t>Lasso</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0.992</v>
+        <v>0.8212</v>
       </c>
       <c r="C24" t="n">
-        <v>0.9921</v>
+        <v>0.8226</v>
       </c>
       <c r="D24" t="n">
-        <v>3.0646</v>
+        <v>14.4859</v>
       </c>
       <c r="E24" t="n">
-        <v>0.1193</v>
+        <v>0.0742</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Lasso</t>
+          <t>LassoLars</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>0.9913</v>
+        <v>0.8212</v>
       </c>
       <c r="C25" t="n">
-        <v>0.9913999999999999</v>
+        <v>0.8226</v>
       </c>
       <c r="D25" t="n">
-        <v>3.189</v>
+        <v>14.4861</v>
       </c>
       <c r="E25" t="n">
-        <v>0.06519999999999999</v>
+        <v>0.0512</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>LassoLars</t>
+          <t>OrthogonalMatchingPursuit</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>0.9913</v>
+        <v>0.8111</v>
       </c>
       <c r="C26" t="n">
-        <v>0.9913999999999999</v>
+        <v>0.8126</v>
       </c>
       <c r="D26" t="n">
-        <v>3.1897</v>
+        <v>14.8901</v>
       </c>
       <c r="E26" t="n">
-        <v>0.0484</v>
+        <v>0.0476</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>PassiveAggressiveRegressor</t>
+          <t>OrthogonalMatchingPursuitCV</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>0.9913</v>
+        <v>0.8111</v>
       </c>
       <c r="C27" t="n">
-        <v>0.9913999999999999</v>
+        <v>0.8126</v>
       </c>
       <c r="D27" t="n">
-        <v>3.1916</v>
+        <v>14.8901</v>
       </c>
       <c r="E27" t="n">
-        <v>0.125</v>
+        <v>0.146</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>KNeighborsRegressor</t>
+          <t>AdaBoostRegressor</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>0.9761</v>
+        <v>0.7881</v>
       </c>
       <c r="C28" t="n">
-        <v>0.9762999999999999</v>
+        <v>0.7897999999999999</v>
       </c>
       <c r="D28" t="n">
-        <v>5.2957</v>
+        <v>15.7697</v>
       </c>
       <c r="E28" t="n">
-        <v>0.9587</v>
+        <v>2.177</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>PoissonRegressor</t>
+          <t>ElasticNet</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0.961</v>
+        <v>0.7627</v>
       </c>
       <c r="C29" t="n">
-        <v>0.9613</v>
+        <v>0.7647</v>
       </c>
       <c r="D29" t="n">
-        <v>6.7634</v>
+        <v>16.6855</v>
       </c>
       <c r="E29" t="n">
-        <v>0.1251</v>
+        <v>0.0557</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>AdaBoostRegressor</t>
+          <t>TweedieRegressor</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>0.9238</v>
+        <v>0.7216</v>
       </c>
       <c r="C30" t="n">
-        <v>0.9244</v>
+        <v>0.7239</v>
       </c>
       <c r="D30" t="n">
-        <v>9.455399999999999</v>
+        <v>18.0736</v>
       </c>
       <c r="E30" t="n">
-        <v>2.352</v>
+        <v>0.06279999999999999</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ElasticNet</t>
+          <t>GammaRegressor</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>0.9161</v>
+        <v>0.7207</v>
       </c>
       <c r="C31" t="n">
-        <v>0.9167999999999999</v>
+        <v>0.723</v>
       </c>
       <c r="D31" t="n">
-        <v>9.921799999999999</v>
+        <v>18.1023</v>
       </c>
       <c r="E31" t="n">
-        <v>0.0489</v>
+        <v>0.0582</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>GammaRegressor</t>
+          <t>NuSVR</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>0.8688</v>
+        <v>0.7128</v>
       </c>
       <c r="C32" t="n">
-        <v>0.8698</v>
+        <v>0.7151</v>
       </c>
       <c r="D32" t="n">
-        <v>12.4093</v>
+        <v>18.3587</v>
       </c>
       <c r="E32" t="n">
-        <v>0.0474</v>
+        <v>61.0871</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>TweedieRegressor</t>
+          <t>SVR</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>0.8661</v>
+        <v>0.7113</v>
       </c>
       <c r="C33" t="n">
-        <v>0.8672</v>
+        <v>0.7137</v>
       </c>
       <c r="D33" t="n">
-        <v>12.536</v>
+        <v>18.4047</v>
       </c>
       <c r="E33" t="n">
-        <v>0.055</v>
+        <v>62.1341</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SVR</t>
+          <t>PassiveAggressiveRegressor</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>0.7754</v>
+        <v>0.5955</v>
       </c>
       <c r="C34" t="n">
-        <v>0.7772</v>
+        <v>0.5988</v>
       </c>
       <c r="D34" t="n">
-        <v>16.235</v>
+        <v>21.7866</v>
       </c>
       <c r="E34" t="n">
-        <v>58.3774</v>
+        <v>0.1155</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>NuSVR</t>
+          <t>RANSACRegressor</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>0.7752</v>
+        <v>0.275</v>
       </c>
       <c r="C35" t="n">
-        <v>0.777</v>
+        <v>0.2809</v>
       </c>
       <c r="D35" t="n">
-        <v>16.2421</v>
+        <v>29.1677</v>
       </c>
       <c r="E35" t="n">
-        <v>68.4477</v>
+        <v>0.2739</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>GaussianProcessRegressor</t>
+          <t>DummyRegressor</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>0.6556999999999999</v>
+        <v>-0.0083</v>
       </c>
       <c r="C36" t="n">
-        <v>0.6585</v>
+        <v>-0</v>
       </c>
       <c r="D36" t="n">
-        <v>20.0993</v>
+        <v>34.3963</v>
       </c>
       <c r="E36" t="n">
-        <v>1689.6609</v>
+        <v>0.0372</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Lars</t>
+          <t>QuantileRegressor</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>0.2595</v>
+        <v>-0.0179</v>
       </c>
       <c r="C37" t="n">
-        <v>0.2656</v>
+        <v>-0.009599999999999999</v>
       </c>
       <c r="D37" t="n">
-        <v>29.4763</v>
+        <v>34.5612</v>
       </c>
       <c r="E37" t="n">
-        <v>0.1779</v>
+        <v>26.4743</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>DummyRegressor</t>
+          <t>GaussianProcessRegressor</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>-0.0083</v>
+        <v>-0.487</v>
       </c>
       <c r="C38" t="n">
-        <v>-0</v>
+        <v>-0.4748</v>
       </c>
       <c r="D38" t="n">
-        <v>34.3963</v>
+        <v>41.7714</v>
       </c>
       <c r="E38" t="n">
-        <v>0.036</v>
+        <v>1874.9665</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>QuantileRegressor</t>
+          <t>Lars</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>-0.018</v>
+        <v>-35573.5988</v>
       </c>
       <c r="C39" t="n">
-        <v>-0.009599999999999999</v>
+        <v>-35282.5604</v>
       </c>
       <c r="D39" t="n">
-        <v>34.5612</v>
+        <v>6460.9386</v>
       </c>
       <c r="E39" t="n">
-        <v>25.4748</v>
+        <v>0.1905</v>
       </c>
     </row>
     <row r="40">
@@ -1172,16 +1172,16 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>-3.454896360262788e+18</v>
+        <v>-3.768817314720178e+18</v>
       </c>
       <c r="C40" t="n">
-        <v>-3.426317542993093e+18</v>
+        <v>-3.737984339688379e+18</v>
       </c>
       <c r="D40" t="n">
-        <v>63668294637.3542</v>
+        <v>66500996208.2966</v>
       </c>
       <c r="E40" t="n">
-        <v>0.0939</v>
+        <v>0.0963</v>
       </c>
     </row>
   </sheetData>

</xml_diff>